<commit_message>
review sheet updated version with last review point solved
</commit_message>
<xml_diff>
--- a/06_Audit/Weekly_Review/QA_Workshop_Review_Sheet.xlsx
+++ b/06_Audit/Weekly_Review/QA_Workshop_Review_Sheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shady gamal\OneDrive\Desktop\QA_Workshop\06_Audit\Weekly_Review\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A7F16E5-DC27-47AF-8F1A-8DBAC384B76B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DAEB7A6-1B0E-4008-927A-7034CBCB7C68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="1545" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="9">
   <si>
     <t>Comment</t>
   </si>
@@ -55,9 +55,6 @@
   </si>
   <si>
     <t>srs is not composed clearly</t>
-  </si>
-  <si>
-    <t>open</t>
   </si>
 </sst>
 </file>
@@ -454,7 +451,7 @@
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">

</xml_diff>